<commit_message>
Rename probo.sh -> probo
</commit_message>
<xml_diff>
--- a/matrix.xlsx
+++ b/matrix.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\workspace\probo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCA1BBF5-BE9F-460F-8A67-8DB435967D0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D57E63B-5575-4443-A473-307D6041B305}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29835" yWindow="3000" windowWidth="21600" windowHeight="13185" xr2:uid="{666122EA-C427-4AFA-9FCF-C46F2029CB39}"/>
+    <workbookView xWindow="31350" yWindow="3390" windowWidth="21600" windowHeight="13185" xr2:uid="{666122EA-C427-4AFA-9FCF-C46F2029CB39}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
--init での conf file 生成を拡充
</commit_message>
<xml_diff>
--- a/matrix.xlsx
+++ b/matrix.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\workspace\probo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D57E63B-5575-4443-A473-307D6041B305}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34F6E85B-8171-4AF2-B197-B249EA914BA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="31350" yWindow="3390" windowWidth="21600" windowHeight="13185" xr2:uid="{666122EA-C427-4AFA-9FCF-C46F2029CB39}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{666122EA-C427-4AFA-9FCF-C46F2029CB39}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="88">
   <si>
     <t>GitLab</t>
     <phoneticPr fontId="1"/>
@@ -179,12 +180,339 @@
     </r>
     <phoneticPr fontId="1"/>
   </si>
+  <si>
+    <t>PROBO_REPORT_TYPE</t>
+  </si>
+  <si>
+    <t>PROBO_FULLSTAT_FILENAME</t>
+  </si>
+  <si>
+    <t>PROBO_FULLSTAT_INSERTION</t>
+  </si>
+  <si>
+    <t>PROBO_PARTSTAT_FILENAME</t>
+  </si>
+  <si>
+    <t>PROBO_PARTSTAT_INSERTION</t>
+  </si>
+  <si>
+    <t>PROBO_BDDAT_FILENAME</t>
+  </si>
+  <si>
+    <t>PROBO_SUMDAT_FILENAME</t>
+  </si>
+  <si>
+    <t>PROBO_SUMDAT_INSERTION</t>
+  </si>
+  <si>
+    <t>PROBO_BDIMG_FILENAME</t>
+  </si>
+  <si>
+    <t>PROBO_BDIMG_WIDTH</t>
+  </si>
+  <si>
+    <t>PROBO_BDIMG_HEIGHT</t>
+  </si>
+  <si>
+    <t>PROBO_BDIMG_BGCLR</t>
+  </si>
+  <si>
+    <t>PROBO_BDIMG_CLR_GUIDE</t>
+  </si>
+  <si>
+    <t>PROBO_BDIMG_CLR_PASSLINE</t>
+  </si>
+  <si>
+    <t>PROBO_BDIMG_CLR_FAILBOX</t>
+  </si>
+  <si>
+    <t>PROBO_SUMIMG_FILENAME</t>
+  </si>
+  <si>
+    <t>PROBO_SUMIMG_WIDTH</t>
+  </si>
+  <si>
+    <t>PROBO_SUMIMG_HEIGHT</t>
+  </si>
+  <si>
+    <t>PROBO_SUMIMG_BGCLR</t>
+  </si>
+  <si>
+    <t>PROBO_SUMIMG_CLR_READY</t>
+  </si>
+  <si>
+    <t>PROBO_SUMIMG_CLR_BLOCK</t>
+  </si>
+  <si>
+    <t>PROBO_SUMIMG_CLR_RUN</t>
+  </si>
+  <si>
+    <t>PROBO_SUMIMG_CLR_PASS</t>
+  </si>
+  <si>
+    <t>PROBO_SUMIMG_CLR_FAIL</t>
+  </si>
+  <si>
+    <t>PROBO_SUMIMG_CLR_REJECT</t>
+  </si>
+  <si>
+    <t>PROBO_SUMIMG_CLR_OTHER</t>
+  </si>
+  <si>
+    <t>PROBO_GRP_FULLSTAT_FILENAME</t>
+  </si>
+  <si>
+    <t>PROBO_GRP_FULLSTAT_INSERTION</t>
+  </si>
+  <si>
+    <t>PROBO_GRP_PARTSTAT_FILENAME</t>
+  </si>
+  <si>
+    <t>PROBO_GRP_PARTSTAT_INSERTION</t>
+  </si>
+  <si>
+    <t>PROBO_GRP_SUMIMG_FILENAME</t>
+  </si>
+  <si>
+    <t>PROBO_BD_STARTDAY</t>
+  </si>
+  <si>
+    <t>PROBO_BD_ENDDAY</t>
+  </si>
+  <si>
+    <t>PROBO_BD_EXEC_PER_DAY</t>
+  </si>
+  <si>
+    <t>PROBO_BD_SCHEDULE</t>
+  </si>
+  <si>
+    <t>markdown</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>gitlab</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>github</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>default</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>REPORT_TYPE</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>----</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>README.md</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>&lt;none&gt;</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>burndown.svg</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>white</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>gray</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>blue</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>red</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>summary.svg</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>#F5F5F5</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>#D2B48C</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>#B0C4DE</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>#FFC1C1</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>#CD9B9B</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>#EEEED1</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>#B0E0E6</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>&lt;auto&gt;</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>summary.data</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>status.full.data</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>status.part.data</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>status.full.txt</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>burndown.data.txt</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>summary.data.txt</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">GNUPLOT </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="游ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>有無のみで制御</t>
+    </r>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">git(hub|lab) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="ＭＳ Ｐゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>か否かで制御</t>
+    </r>
+    <rPh sb="14" eb="15">
+      <t>イナ</t>
+    </rPh>
+    <rPh sb="17" eb="19">
+      <t>セイギョ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">git(hub|lab) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="ＭＳ Ｐゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>か否か</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Courier New"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> &amp;&amp; GNUPLOT </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="ＭＳ Ｐゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>有無で制御</t>
+    </r>
+    <rPh sb="14" eb="15">
+      <t>イナ</t>
+    </rPh>
+    <rPh sb="28" eb="30">
+      <t>ウム</t>
+    </rPh>
+    <rPh sb="31" eb="33">
+      <t>セイギョ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>自動</t>
+    <rPh sb="0" eb="2">
+      <t>ジドウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>常になし</t>
+    <rPh sb="0" eb="1">
+      <t>ツネ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>raw か否かで制御</t>
+    <rPh sb="5" eb="6">
+      <t>イナ</t>
+    </rPh>
+    <rPh sb="8" eb="10">
+      <t>セイギョ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>report.md</t>
+    <phoneticPr fontId="1"/>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -225,8 +553,41 @@
       <charset val="128"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Courier New"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Courier New"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Courier New"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="游ゴシック"/>
+      <family val="3"/>
+      <charset val="128"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="ＭＳ Ｐゴシック"/>
+      <family val="3"/>
+      <charset val="128"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -236,6 +597,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -312,7 +685,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -337,6 +710,15 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -351,6 +733,27 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -695,18 +1098,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:6" x14ac:dyDescent="0.4">
-      <c r="B2" s="9"/>
-      <c r="C2" s="8" t="s">
+      <c r="B2" s="12"/>
+      <c r="C2" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="11" t="s">
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
+      <c r="F2" s="14" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="3" spans="2:6" x14ac:dyDescent="0.4">
-      <c r="B3" s="10"/>
+      <c r="B3" s="13"/>
       <c r="C3" s="2" t="s">
         <v>0</v>
       </c>
@@ -716,7 +1119,7 @@
       <c r="E3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="F3" s="12"/>
+      <c r="F3" s="15"/>
     </row>
     <row r="4" spans="2:6" ht="47.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B4" s="3" t="s">
@@ -817,4 +1220,941 @@
   <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3C02FCF-358A-487F-905B-F50860278A3A}">
+  <dimension ref="A1:H46"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="1" width="35.75" style="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="7" width="21.125" style="8" customWidth="1"/>
+    <col min="8" max="16384" width="9" style="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A1" s="16"/>
+      <c r="B1" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+    </row>
+    <row r="2" spans="1:8" ht="15.75" x14ac:dyDescent="0.4">
+      <c r="A2" s="16"/>
+      <c r="B2" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="E2" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="F2" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="G2" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A3" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="18" t="s">
+        <v>53</v>
+      </c>
+      <c r="D3" s="18" t="s">
+        <v>53</v>
+      </c>
+      <c r="E3" s="18" t="s">
+        <v>53</v>
+      </c>
+      <c r="F3" s="18" t="s">
+        <v>53</v>
+      </c>
+      <c r="G3" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="H3" s="22" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A4" s="20"/>
+      <c r="B4" s="21"/>
+      <c r="C4" s="21"/>
+      <c r="D4" s="21"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="21"/>
+      <c r="G4" s="21"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A5" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="C5" s="18" t="s">
+        <v>87</v>
+      </c>
+      <c r="D5" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="E5" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="F5" s="18" t="s">
+        <v>76</v>
+      </c>
+      <c r="G5" s="18"/>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A6" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="18">
+        <v>0</v>
+      </c>
+      <c r="C6" s="18">
+        <v>1</v>
+      </c>
+      <c r="D6" s="18">
+        <v>1</v>
+      </c>
+      <c r="E6" s="18">
+        <v>1</v>
+      </c>
+      <c r="F6" s="18">
+        <v>0</v>
+      </c>
+      <c r="G6" s="18"/>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A7" s="20"/>
+      <c r="B7" s="21"/>
+      <c r="C7" s="21"/>
+      <c r="D7" s="21"/>
+      <c r="E7" s="21"/>
+      <c r="F7" s="21"/>
+      <c r="G7" s="21"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A8" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="C8" s="18" t="s">
+        <v>87</v>
+      </c>
+      <c r="D8" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="E8" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="F8" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="G8" s="18"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A9" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" s="18">
+        <v>0</v>
+      </c>
+      <c r="C9" s="18">
+        <v>1</v>
+      </c>
+      <c r="D9" s="18">
+        <v>1</v>
+      </c>
+      <c r="E9" s="18">
+        <v>1</v>
+      </c>
+      <c r="F9" s="18">
+        <v>0</v>
+      </c>
+      <c r="G9" s="18"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A10" s="20"/>
+      <c r="B10" s="21"/>
+      <c r="C10" s="21"/>
+      <c r="D10" s="21"/>
+      <c r="E10" s="21"/>
+      <c r="F10" s="21"/>
+      <c r="G10" s="21"/>
+    </row>
+    <row r="11" spans="1:8" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A11" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B11" s="18" t="s">
+        <v>79</v>
+      </c>
+      <c r="C11" s="18"/>
+      <c r="D11" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="E11" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="F11" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="G11" s="18"/>
+      <c r="H11" s="8" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A12" s="20"/>
+      <c r="B12" s="21"/>
+      <c r="C12" s="21"/>
+      <c r="D12" s="21"/>
+      <c r="E12" s="21"/>
+      <c r="F12" s="21"/>
+      <c r="G12" s="21"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A13" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="B13" s="18" t="s">
+        <v>80</v>
+      </c>
+      <c r="C13" s="18" t="s">
+        <v>87</v>
+      </c>
+      <c r="D13" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="E13" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="F13" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="G13" s="18"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A14" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="B14" s="18">
+        <v>0</v>
+      </c>
+      <c r="C14" s="18">
+        <v>1</v>
+      </c>
+      <c r="D14" s="18">
+        <v>1</v>
+      </c>
+      <c r="E14" s="18">
+        <v>1</v>
+      </c>
+      <c r="F14" s="18">
+        <v>0</v>
+      </c>
+      <c r="G14" s="18"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A15" s="20"/>
+      <c r="B15" s="21"/>
+      <c r="C15" s="21"/>
+      <c r="D15" s="21"/>
+      <c r="E15" s="21"/>
+      <c r="F15" s="21"/>
+      <c r="G15" s="21"/>
+    </row>
+    <row r="16" spans="1:8" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A16" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="B16" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="C16" s="18"/>
+      <c r="D16" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="E16" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="F16" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="G16" s="18"/>
+      <c r="H16" s="8" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A17" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="B17" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="C17" s="18"/>
+      <c r="D17" s="18">
+        <v>800</v>
+      </c>
+      <c r="E17" s="18">
+        <v>800</v>
+      </c>
+      <c r="F17" s="18">
+        <v>800</v>
+      </c>
+      <c r="G17" s="18"/>
+      <c r="H17" s="8" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A18" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="B18" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="C18" s="18"/>
+      <c r="D18" s="18">
+        <v>400</v>
+      </c>
+      <c r="E18" s="18">
+        <v>400</v>
+      </c>
+      <c r="F18" s="18">
+        <v>400</v>
+      </c>
+      <c r="G18" s="18"/>
+      <c r="H18" s="8" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A19" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="B19" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="C19" s="18"/>
+      <c r="D19" s="18" t="s">
+        <v>62</v>
+      </c>
+      <c r="E19" s="18" t="s">
+        <v>62</v>
+      </c>
+      <c r="F19" s="18" t="s">
+        <v>62</v>
+      </c>
+      <c r="G19" s="18"/>
+      <c r="H19" s="8" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A20" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="B20" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="C20" s="18"/>
+      <c r="D20" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="E20" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="F20" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="G20" s="18"/>
+      <c r="H20" s="8" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A21" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B21" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="C21" s="18"/>
+      <c r="D21" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="E21" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="F21" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="G21" s="18"/>
+      <c r="H21" s="8" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A22" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="B22" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="C22" s="18"/>
+      <c r="D22" s="18" t="s">
+        <v>65</v>
+      </c>
+      <c r="E22" s="18" t="s">
+        <v>65</v>
+      </c>
+      <c r="F22" s="18" t="s">
+        <v>65</v>
+      </c>
+      <c r="G22" s="18"/>
+      <c r="H22" s="8" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A23" s="20"/>
+      <c r="B23" s="21"/>
+      <c r="C23" s="21"/>
+      <c r="D23" s="21"/>
+      <c r="E23" s="21"/>
+      <c r="F23" s="21"/>
+      <c r="G23" s="21"/>
+    </row>
+    <row r="24" spans="1:8" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A24" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="B24" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="C24" s="18"/>
+      <c r="D24" s="18" t="s">
+        <v>66</v>
+      </c>
+      <c r="E24" s="18" t="s">
+        <v>66</v>
+      </c>
+      <c r="F24" s="18" t="s">
+        <v>66</v>
+      </c>
+      <c r="G24" s="18"/>
+      <c r="H24" s="8" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A25" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="B25" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="C25" s="18"/>
+      <c r="D25" s="18">
+        <v>500</v>
+      </c>
+      <c r="E25" s="18">
+        <v>500</v>
+      </c>
+      <c r="F25" s="18">
+        <v>500</v>
+      </c>
+      <c r="G25" s="18"/>
+      <c r="H25" s="8" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A26" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="B26" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="C26" s="18"/>
+      <c r="D26" s="18">
+        <v>400</v>
+      </c>
+      <c r="E26" s="18">
+        <v>400</v>
+      </c>
+      <c r="F26" s="18">
+        <v>400</v>
+      </c>
+      <c r="G26" s="18"/>
+      <c r="H26" s="8" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A27" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="B27" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="C27" s="18"/>
+      <c r="D27" s="18" t="s">
+        <v>62</v>
+      </c>
+      <c r="E27" s="18" t="s">
+        <v>62</v>
+      </c>
+      <c r="F27" s="18" t="s">
+        <v>62</v>
+      </c>
+      <c r="G27" s="18"/>
+      <c r="H27" s="8" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A28" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="B28" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="C28" s="18"/>
+      <c r="D28" s="18" t="s">
+        <v>67</v>
+      </c>
+      <c r="E28" s="18" t="s">
+        <v>67</v>
+      </c>
+      <c r="F28" s="18" t="s">
+        <v>67</v>
+      </c>
+      <c r="G28" s="18"/>
+      <c r="H28" s="8" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A29" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="B29" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="C29" s="18"/>
+      <c r="D29" s="18" t="s">
+        <v>68</v>
+      </c>
+      <c r="E29" s="18" t="s">
+        <v>68</v>
+      </c>
+      <c r="F29" s="18" t="s">
+        <v>68</v>
+      </c>
+      <c r="G29" s="18"/>
+      <c r="H29" s="8" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A30" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="B30" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="C30" s="18"/>
+      <c r="D30" s="18" t="s">
+        <v>69</v>
+      </c>
+      <c r="E30" s="18" t="s">
+        <v>69</v>
+      </c>
+      <c r="F30" s="18" t="s">
+        <v>69</v>
+      </c>
+      <c r="G30" s="18"/>
+      <c r="H30" s="8" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A31" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="B31" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="C31" s="18"/>
+      <c r="D31" s="18" t="s">
+        <v>73</v>
+      </c>
+      <c r="E31" s="18" t="s">
+        <v>73</v>
+      </c>
+      <c r="F31" s="18" t="s">
+        <v>73</v>
+      </c>
+      <c r="G31" s="18"/>
+      <c r="H31" s="8" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A32" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="B32" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="C32" s="18"/>
+      <c r="D32" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="E32" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="F32" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="G32" s="18"/>
+      <c r="H32" s="8" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A33" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="B33" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="C33" s="18"/>
+      <c r="D33" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="E33" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="F33" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="G33" s="18"/>
+      <c r="H33" s="8" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A34" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="B34" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="C34" s="18"/>
+      <c r="D34" s="18" t="s">
+        <v>72</v>
+      </c>
+      <c r="E34" s="18" t="s">
+        <v>72</v>
+      </c>
+      <c r="F34" s="18" t="s">
+        <v>72</v>
+      </c>
+      <c r="G34" s="18"/>
+      <c r="H34" s="8" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A35" s="20"/>
+      <c r="B35" s="21"/>
+      <c r="C35" s="21"/>
+      <c r="D35" s="21"/>
+      <c r="E35" s="21"/>
+      <c r="F35" s="21"/>
+      <c r="G35" s="21"/>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A36" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="B36" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="C36" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="D36" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="E36" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="F36" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="G36" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="H36" s="8" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A37" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="B37" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="C37" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="D37" s="18">
+        <v>1</v>
+      </c>
+      <c r="E37" s="18">
+        <v>1</v>
+      </c>
+      <c r="F37" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="G37" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="H37" s="8" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A38" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="B38" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="C38" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="D38" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="E38" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="F38" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="G38" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="H38" s="8" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A39" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="B39" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="C39" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="D39" s="18">
+        <v>1</v>
+      </c>
+      <c r="E39" s="18">
+        <v>1</v>
+      </c>
+      <c r="F39" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="G39" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="H39" s="8" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A40" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="B40" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="C40" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="D40" s="18" t="s">
+        <v>66</v>
+      </c>
+      <c r="E40" s="18" t="s">
+        <v>66</v>
+      </c>
+      <c r="F40" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="G40" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="H40" s="8" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A41" s="20"/>
+      <c r="B41" s="21"/>
+      <c r="C41" s="21"/>
+      <c r="D41" s="21"/>
+      <c r="E41" s="21"/>
+      <c r="F41" s="21"/>
+      <c r="G41" s="21"/>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A42" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="B42" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="C42" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="D42" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="E42" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="F42" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="G42" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="H42" s="22" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A43" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="B43" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="C43" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="D43" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="E43" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="F43" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="G43" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="H43" s="22" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A44" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="B44" s="18">
+        <v>10</v>
+      </c>
+      <c r="C44" s="18">
+        <v>10</v>
+      </c>
+      <c r="D44" s="18">
+        <v>10</v>
+      </c>
+      <c r="E44" s="18">
+        <v>10</v>
+      </c>
+      <c r="F44" s="18">
+        <v>10</v>
+      </c>
+      <c r="G44" s="18">
+        <v>10</v>
+      </c>
+      <c r="H44" s="22" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A45" s="20"/>
+      <c r="B45" s="21"/>
+      <c r="C45" s="21"/>
+      <c r="D45" s="21"/>
+      <c r="E45" s="21"/>
+      <c r="F45" s="21"/>
+      <c r="G45" s="21"/>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.4">
+      <c r="A46" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="B46" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="C46" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="D46" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="E46" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="F46" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="G46" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="H46" s="22" t="s">
+        <v>85</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B1:G1"/>
+    <mergeCell ref="A1:A2"/>
+  </mergeCells>
+  <phoneticPr fontId="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>